<commit_message>
First draft of Stage 5: Enriched Dataset Collection. Also switch to Qwen
</commit_message>
<xml_diff>
--- a/data/enriched_matches.xlsx
+++ b/data/enriched_matches.xlsx
@@ -1,37 +1,140 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pmzdjc/Documents/Personal/Football Match Memory Enricher/data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_7173F2438AA77123ADC3BF982912A919F0203680" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="matches" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Matches" sheetId="1" r:id="rId1"/>
+    <sheet name="Top Scorers" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+  <si>
+    <t>home team</t>
+  </si>
+  <si>
+    <t>home manager</t>
+  </si>
+  <si>
+    <t>home score</t>
+  </si>
+  <si>
+    <t>away team</t>
+  </si>
+  <si>
+    <t>away manager</t>
+  </si>
+  <si>
+    <t>away score</t>
+  </si>
+  <si>
+    <t>goals_summary</t>
+  </si>
+  <si>
+    <t>Manchester United</t>
+  </si>
+  <si>
+    <t>Ruben Amorim</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Brighton</t>
+  </si>
+  <si>
+    <t>Fabian Hurzeler</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Matheus Cunha (24), Casemiro (34), Bryan Mbeumo (61), Bryan Mbeumo (96), Danny Welbeck (74), Charalampos Kostoulas (96)</t>
+  </si>
+  <si>
+    <t>Bournemouth</t>
+  </si>
+  <si>
+    <t>Andoni Iraola</t>
+  </si>
+  <si>
+    <t>Semenyo (13), Bruno Fernandes (40), Matheus Cunha (44), Eli Junior Kroupi (45+1), Evanilson (46), Marcus Tavernier (48), Bruno Fernandes (77), Eli Junior Kroupi (84)</t>
+  </si>
+  <si>
+    <t>Rank</t>
+  </si>
+  <si>
+    <t>Player</t>
+  </si>
+  <si>
+    <t>Goals Seen Live</t>
+  </si>
+  <si>
+    <t>Bruno Fernandes</t>
+  </si>
+  <si>
+    <t>Bryan Mbeumo</t>
+  </si>
+  <si>
+    <t>Eli Junior Kroupi</t>
+  </si>
+  <si>
+    <t>Matheus Cunha</t>
+  </si>
+  <si>
+    <t>Casemiro</t>
+  </si>
+  <si>
+    <t>Charalampos Kostoulas</t>
+  </si>
+  <si>
+    <t>Danny Welbeck</t>
+  </si>
+  <si>
+    <t>Evanilson</t>
+  </si>
+  <si>
+    <t>Marcus Tavernier</t>
+  </si>
+  <si>
+    <t>Semenyo</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,93 +149,43 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -420,29 +473,208 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>home_manager</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Ruben Amorim</t>
-        </is>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>5</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>5</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Pipeline applied to full dataset
</commit_message>
<xml_diff>
--- a/data/enriched_matches.xlsx
+++ b/data/enriched_matches.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,27 +479,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ruben Amorim</t>
+          <t>Sir Alex Ferguson</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Brighton</t>
+          <t>Birmingham</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Fabian Hurzeler</t>
+          <t>Alex McLeish</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -509,7 +509,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Matheus Cunha (24th), Casemiro (34th), Bryan Mbeumo (61st), Danny Welbeck (74th), Bryan Mbeumo (90+6th), Charalampos Kostoulas (90+3rd)</t>
+          <t>Carlos Tevez (25)</t>
         </is>
       </c>
     </row>
@@ -521,37 +521,819 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Sir Alex Ferguson</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Hull</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Phil Brown</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Old Trafford</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Cristiano Ronaldo (3), Michael Carrick (29), Cristiano Ronaldo (44), Nemanja Vidic (57), Bernard Mendy (75), Geovanni (90)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Remi Garde</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Wycombe</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Gareth Ainsworth</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Villa Park</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Ciaran Clark (75'), Idrissa Gueye (90')</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Man United</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Jose Mourinho</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Celta Vigo</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Old Trafford</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Marcus Rashford (67)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Man United</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Jose Mourinho</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Bournemouth</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Eddie Howe</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Old Trafford</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Romelu Lukaku (25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Man United</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ole Gunnar Solskjaer</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Brighton</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Graham Potter</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Old Trafford</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Davy Propper (19), Andreas Pereira (), Marcus Rashford ()</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Man United</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Ole Gunnar Solskjær</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Dean Smith</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Old Trafford</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Jack Grealish (N/A), Marcus Rashford (N/A), Victor Lindelöf (N/A), Tyrone Mings (N/A)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Leicester</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Brendan Rodgers</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Norwich</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Daniel Farke</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>King Power Stadium</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Teemu Pukki (25th), Tim Krul (37th)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Man United</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Ole Gunnar Solskjær</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Nigel Pearson</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Old Trafford</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Bruno Fernandes (unknown), Anthony Martial (unknown), Mason Greenwood (unknown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Norwich</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Dean Smith</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Man United</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Ralf Rangnick</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Carrow Road</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Cristiano Ronaldo (75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Wolves</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Bruno Lage</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Norwich</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Dean Smith</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Molineux</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Kenny McLean (45'+1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Steven Gerrard</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Norwich</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Dean Smith</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Villa Park</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Ollie Watkins (first half), Danny Ings (stoppage time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Wolves</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Bruno Lage</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Norwich</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Dean Smith</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Molineax</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Teemu Pukki (37th), Rayan Aït-Nouri (55th)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Man United</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Erik ten Hag</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Unai Emery</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Old Trafford</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Anthony Martial (49'), Marcus Rashford (67'), Bruno Fernandes (78'), Scott McTominay (90'+1'), Ollie Watkins (48'), Diogo Dalot (61')</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>West Brown</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Carlos Corberan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Norwich</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>David Wagner</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Hawthorns</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Josh Sargent (41), Conor Townsend (45+1), Jed Wallace ()</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Man United</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Emirates Stadium</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Marcus Rashford (unknown), Martin Ødegaard (unknown), Declan Rice (unknown), Gabriel Jesus (unknown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>West Ham</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>David Moyes</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Mikel Arteta</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Olympic Stadium</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>William Saliba (32), Bukayo Saka (41), Gabriel (44), Leandro Trossard (45+2), Bukayo Saka (63), Declan Rice (66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Chelsea</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Mauricio Pochettino</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Man United</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Erik ten Hag</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Stamford Bridge</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Cole Palmer (6), Cole Palmer (99), Alejandro Garnacho (), Bruno Fernandes (), Conor Gallagher ()</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Chelsea</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Enzo Maresca</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Barrow</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Stamford Bridge</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Christopher Nkunku (8'), Christopher Nkunku (15'), Paul Farman (28'), Pedro Neto (48'), Christopher Nkunku (75')</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Man United</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>Ruben Amorim</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Brighton</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Fabian Hurzeler</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Old Trafford</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Matheus Cunha (24), Casemiro (34), Bryan Mbeumo (61), Danny Welbeck (74), Charalampos Kostoulas (90+2), Bryan Mbeumo (90+7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Man United</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Ruben Amorim</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
         <is>
           <t>Bournemouth</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Andoni Iraola</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>Old Trafford</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Amad Diallo (13), Casemiro (40), Bruno Fernandes (75), Matheus Cunha (77), Evanilson (82), Marcus Tavernier (84), Eli Junior Kroupi (90)</t>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Amad Diallo (13), Evanilson (46), Marcus Tavernier (52), Bruno Fernandes (78), Matheus Cunha (80), Eli Junior Kroupi (84)</t>
         </is>
       </c>
     </row>
@@ -566,7 +1348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -592,127 +1374,660 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bryan Mbeumo</t>
+          <t>Marcus Rashford</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Casemiro</t>
+          <t>Bruno Fernandes</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Matheus Cunha</t>
+          <t>Christopher Nkunku</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Amad Diallo</t>
+          <t>Cristiano Ronaldo</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Bruno Fernandes</t>
+          <t>Anthony Martial</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Charalampos Kostoulas</t>
+          <t>Bryan Mbeumo</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Danny Welbeck</t>
+          <t>Bukayo Saka</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Eli Junior Kroupi</t>
+          <t>Cole Palmer</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Evanilson</t>
+          <t>Declan Rice</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>Matheus Cunha</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Ollie Watkins</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Teemu Pukki</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Alejandro Garnacho</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Amad Diallo</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Andreas Pereira</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Bernard Mendy</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Carlos Tevez</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>13</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Casemiro</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>13</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Charalampos Kostoulas</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>13</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Ciaran Clark</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>13</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Conor Gallagher</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>13</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Conor Townsend</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>13</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Danny Ings</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>13</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Danny Welbeck</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>13</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Davy Propper</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>13</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Diogo Dalot</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>13</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Eli Junior Kroupi</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>13</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Evanilson</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>13</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Gabriel</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>13</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Gabriel Jesus</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>13</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Geovanni</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>13</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Idrissa Gueye</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>13</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Jack Grealish</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>13</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Jed Wallace</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>13</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Josh Sargent</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>13</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Kenny McLean</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>13</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Leandro Trossard</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>13</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
           <t>Marcus Tavernier</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>13</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Martin Ødegaard</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>13</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Mason Greenwood</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>13</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Michael Carrick</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>13</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Nemanja Vidic</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>13</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Paul Farman</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>13</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Pedro Neto</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>13</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Rayan Aït-Nouri</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>13</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Romelu Lukaku</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>13</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Scott McTominay</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>13</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Tim Krul</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>13</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Tyrone Mings</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>13</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Victor Lindelöf</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>13</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>William Saliba</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>